<commit_message>
auto commit by win-upload.bat
</commit_message>
<xml_diff>
--- a/COMPONENTS/list.xlsx
+++ b/COMPONENTS/list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJ\ArduinoNode\COMPONENTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A587CDCB-369C-484B-8E23-A56E41E17ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA474A2F-EA83-49A0-B6A6-BE4CCD5C03BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0C3D26CF-E483-42EF-A99D-67E985857491}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{0C3D26CF-E483-42EF-A99D-67E985857491}"/>
   </bookViews>
   <sheets>
     <sheet name="Original Plan" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
   <si>
     <t>Item</t>
   </si>
@@ -736,9 +736,6 @@
     <t>3D Printed Case</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandisk </t>
-  </si>
-  <si>
     <t xml:space="preserve">nrf24l01 </t>
   </si>
   <si>
@@ -758,13 +755,52 @@
   </si>
   <si>
     <t>RGB LED Matrix (module and wire)</t>
+  </si>
+  <si>
+    <t>Wiring</t>
+  </si>
+  <si>
+    <t>Dupont Wires</t>
+  </si>
+  <si>
+    <t>cloth tape</t>
+  </si>
+  <si>
+    <t>Screw</t>
+  </si>
+  <si>
+    <t>Battery Holder</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Multimeter</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>Nut</t>
+  </si>
+  <si>
+    <t>To connect arduino / battery holder to the printed board</t>
+  </si>
+  <si>
+    <t>hex standoff</t>
+  </si>
+  <si>
+    <t>0.2/g</t>
+  </si>
+  <si>
+    <t>Hex Standoff</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -823,8 +859,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -849,6 +891,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -863,7 +911,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -874,13 +922,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -889,7 +935,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1292,12 +1344,12 @@
       <c r="F2" s="4">
         <v>735</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1315,7 +1367,7 @@
       <c r="F3" s="4">
         <v>235.2</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H3" s="1" t="s">
@@ -1324,7 +1376,7 @@
       <c r="I3" s="1">
         <v>165</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1347,7 +1399,7 @@
       <c r="F4" s="1">
         <v>9.8000000000000007</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1370,7 +1422,7 @@
       <c r="F5" s="4">
         <v>18.62</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1393,7 +1445,7 @@
       <c r="F6" s="4">
         <v>10.78</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1416,7 +1468,7 @@
       <c r="F7" s="4">
         <v>10.78</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1439,7 +1491,7 @@
       <c r="F8" s="4">
         <v>2.94</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
@@ -1448,7 +1500,7 @@
       <c r="I8" s="1">
         <v>24.8</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1471,7 +1523,16 @@
       <c r="F9" s="1">
         <v>48</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="1">
+        <v>33</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1485,16 +1546,16 @@
       <c r="C10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <v>3.02</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="8">
         <v>3.02</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H10" s="1" t="s">
@@ -1508,7 +1569,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="9" t="s">
         <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -1523,7 +1584,7 @@
       <c r="E11" s="1">
         <v>9</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="4">
         <v>9.31</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -1540,7 +1601,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="17" t="s">
         <v>35</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1552,11 +1613,17 @@
       <c r="D12" s="7" t="s">
         <v>38</v>
       </c>
+      <c r="E12" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="G12" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="17" t="s">
+        <v>72</v>
+      </c>
       <c r="B13" s="1" t="s">
         <v>40</v>
       </c>
@@ -1569,61 +1636,79 @@
       <c r="E13" s="1">
         <v>78</v>
       </c>
+      <c r="F13" s="1">
+        <v>78</v>
+      </c>
       <c r="G13" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="B14" s="11" t="s">
+      <c r="A14" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>9.5299999999999994</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13" t="s">
+      <c r="F14" s="1">
+        <v>9.5299999999999994</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+      <c r="A15" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="10">
         <v>9.31</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="13" t="s">
+      <c r="F15" s="1">
+        <v>9.31</v>
+      </c>
+      <c r="G15" s="11" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="10">
         <v>39.799999999999997</v>
       </c>
-      <c r="F16" s="12"/>
-      <c r="G16" s="13" t="s">
+      <c r="F16" s="16">
+        <v>38.130000000000003</v>
+      </c>
+      <c r="G16" s="11" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1648,217 +1733,315 @@
     <hyperlink ref="G14" r:id="rId17" display="https://detail.tmall.com/item.htm?id=41254478179&amp;ns=1&amp;pisk=gqUnFNMNanAW2B_cRdgCcEkZvBsOz2gSA8L-e4HPbAk6J0kRA8mueRizJ2FLIYyYEbULyzq6rSN7J6gRO2NIP4WAHZ3uOWgWpeLWYymw7XFw8pkFXVWp_4bOHZQYsMlIy5WYJIA3UXGvz4oE4AuZCbceT0yrbFlSQely8bJNsAGrzX-E4NPZibteL4yr_VloiU8y8UuwQXHZU4uzU55iZbQvzx4z5PWMjwi0a8xLBXmn3WkUwb4wYb-QiAvBpPqG0xFeVU8zSXmUPLoWWU3u4SZozVfFzWwxC0kQQNLnr5lunj2HQO0zsyambyW6r2UQToozuTtznyNUzc4RBhD4X5Za-cRyP0UILJl4ONfa9mMnJP32QTGgbSwSgDv9Y-PTMyi_rtvZFkhj7X2PuOjzah-2kQ8S__UwV3iE1fDxxccMUfMR0D1GsnsIYfGdH1fMV3iE1XBAs1xfADls9tC..&amp;priceTId=2147843917384670564475028edfef&amp;skuId=5363149407088&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%22ec9d2b1fda83dc21e35b93883a6eaced%22%7D&amp;xxc=ad_ztc" xr:uid="{B2BFBBBB-D659-4D0D-B759-A2D78175E2DF}"/>
     <hyperlink ref="G15" r:id="rId18" display="https://detail.tmall.com/item.htm?id=41254478179&amp;ns=1&amp;pisk=gqUnFNMNanAW2B_cRdgCcEkZvBsOz2gSA8L-e4HPbAk6J0kRA8mueRizJ2FLIYyYEbULyzq6rSN7J6gRO2NIP4WAHZ3uOWgWpeLWYymw7XFw8pkFXVWp_4bOHZQYsMlIy5WYJIA3UXGvz4oE4AuZCbceT0yrbFlSQely8bJNsAGrzX-E4NPZibteL4yr_VloiU8y8UuwQXHZU4uzU55iZbQvzx4z5PWMjwi0a8xLBXmn3WkUwb4wYb-QiAvBpPqG0xFeVU8zSXmUPLoWWU3u4SZozVfFzWwxC0kQQNLnr5lunj2HQO0zsyambyW6r2UQToozuTtznyNUzc4RBhD4X5Za-cRyP0UILJl4ONfa9mMnJP32QTGgbSwSgDv9Y-PTMyi_rtvZFkhj7X2PuOjzah-2kQ8S__UwV3iE1fDxxccMUfMR0D1GsnsIYfGdH1fMV3iE1XBAs1xfADls9tC..&amp;priceTId=2147843917384670564475028edfef&amp;skuId=5627773561514&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%22ec9d2b1fda83dc21e35b93883a6eaced%22%7D&amp;xxc=ad_ztc" xr:uid="{A330A296-4CAF-4510-BAE6-7C44882320A4}"/>
     <hyperlink ref="G16" r:id="rId19" display="https://item.taobao.com/item.htm?app=chrome&amp;bxsign=scd4fgYf5iF5OAmJicIo8iDGaUsRWCKvhd72ySfn57pRrBT2pPAYhLKu9gtqqdEx21nKi6ZyseOSsTa8eiwPArHIefizS99FVtzGhG4EdHu0E4hIZCd1MlLQ-RQyEYvWfih&amp;cpp=1&amp;id=732795303962&amp;price=39.8&amp;shareUniqueId=30526150185&amp;share_crt_v=1&amp;shareurl=true&amp;short_name=h.TIfWRzLOj3Nt6rB&amp;skuId=5244345319018&amp;sourceType=item&amp;sp_tk=QTdEVmVpejVhRWU%3D&amp;spm=a2159r.13376460.0.0&amp;suid=C52028D3-13D5-4AB6-AA7D-4C88B1CD3E97&amp;tbSocialPopKey=shareItem&amp;tk=A7DVeiz5aEe&amp;un=da9398d2eb10733dd327b29a79c3809c&amp;un_site=0&amp;ut_sk=1.YQ%2BEdxFco9wDAEpcPBtvBZKC_21380790_1739955800795.Copy.1&amp;wxsign=tbwXAIHPmVF8CbhHdEFpioiPtL818gIgppBaQP38PexM2Q_7iFa1yDdkb90jgKVo8bilX2rQDMmXzgsvPUxqG_mWRxT47fHLuJAztlHa36I7eHamCer6-S_fDEkPlJImFh5" xr:uid="{36DB8C7F-42E0-4C5B-B8C6-40F795E4913E}"/>
+    <hyperlink ref="J9" r:id="rId20" xr:uid="{3C3FE6F1-DA39-43AC-9836-B5FDDE5C8DA2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId20"/>
+  <pageSetup orientation="portrait" r:id="rId21"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82D55E43-80C5-42C3-9768-6336FAD35EF4}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.81640625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="24.1796875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="29.26953125" style="14" customWidth="1"/>
-    <col min="4" max="4" width="23.90625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="34.26953125" style="14" customWidth="1"/>
-    <col min="6" max="6" width="33.54296875" style="14" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="14"/>
+    <col min="1" max="1" width="38.81640625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="24.1796875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="45.6328125" style="12" customWidth="1"/>
+    <col min="4" max="4" width="34.26953125" style="12" customWidth="1"/>
+    <col min="5" max="5" width="33.54296875" style="12" customWidth="1"/>
+    <col min="6" max="16384" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:5" s="15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="14" t="s">
+      <c r="D1" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="14" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="E1" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="14">
+      <c r="D2" s="12">
         <v>165</v>
       </c>
-      <c r="F2" s="14" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="E2" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="14">
+      <c r="D3" s="12">
         <v>9.8000000000000007</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="E3" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="12">
+        <v>10.78</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="12">
+        <v>18.62</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="12">
+        <v>12</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="12">
+        <v>8</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="14">
-        <v>10.78</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="14">
-        <v>18.62</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="14" t="s">
+      <c r="B8" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="12">
+        <v>28.9</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="1">
+        <v>24.8</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="12">
+        <v>48</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="12">
+        <v>116</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="12">
+        <v>2.86</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="12">
+        <v>3.07</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="12">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="14">
-        <v>12</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="14">
-        <v>8</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="14">
-        <v>28.9</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="14">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>65</v>
+      <c r="C15" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" s="12">
+        <v>32.5</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="12">
+        <v>7</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{5B37F600-9DE2-4AEA-96E7-A279D6B80EDB}"/>
-    <hyperlink ref="F3" r:id="rId2" display="https://detail.tmall.com/item.htm?abbucket=6&amp;id=663358716903&amp;pisk=gSEiq3GF3UvffHPJ6Wo1PT7ND-QKCdijOSKxMmhV8XlIXPLOCjz3FWXsDSeqiSVKOlBsMOO0i-2i7Akq7D-ECYJw0fy2nxPKbqatMfhmm-Nlp_IR2Rwscq5RwgnjxJCqVFl20IHeLxmmQlqGbiyscm5Dpn7RqRNPWXPo3xkFKxHv0APq_XlEOxD2QSlZ8Bkjhml4gSuETxMj3Fl2bB8EOYL2bfkwLBkxedlq_SyFKxGEgbZ2bbr4Ak5htVmzcY4uxA0iaJbB0nfnQQhuQ1tD0k4nSb--tn-4xA2dpUhkYilzPWzU7zvwvqnIt8MgGgtsbq4asvocmHog1Rrq-oCpsvaasku0vt_sdPy3m4ZfhFhTRS0uj2vfTviar5lLgKx8GcDSkrmcApGaPyFaYm9JRcU8eogzbGAS94M0ZYVMsgzy8U-J3nMFHk8XlVkIKb3i-vA2pFmSd9XHPmgZdACRK9YXhVkIK7WhKUNj7vMt7&amp;rn=3f9c2948bd3255c25dbbba65f1bf9b72&amp;spm=a1z10.5-b.w4011-25295428345.45.7ca8289cLqsyZo" xr:uid="{95147A8D-CAF1-4545-9FE2-3B467BD86C28}"/>
-    <hyperlink ref="F4" r:id="rId3" display="https://detail.tmall.com/item.htm?abbucket=6&amp;id=745189429142&amp;pisk=gCQxbx9jIDAXfaL3orZksBOSv2PuKNC2wt5ISdvmfTBRh9hcmKf61NBGFFx_3EbOeO6tSibDoha6etgMmNCZWC11QSJggufVgF8_KJYT-s5q15em-ZnjP01yOjO_qnwumOp3KJ43WoGWW-ehnDLCn0OpOFOXfdT7wCdXGFtXc3NJ1CDXCK61N7py_Ig6CFiWNBAjcFgXC4TWgI361mtXN39y1F91CFG4c-p-Gd0OvjLnPfZPpVg1yIK7xs95COFMGndAMLeQdaUeDp1XeVwEYk-9hB_QEmRpDOK5r1cnS3ffYORChxwv5_ddpBBYjfJAV6bDagytXpI1iMS14R3phMfFYhQ0K0fWlKKeLglTwFBPAHQy7filghOd3E_bExL9yB-GXt2r5KjdNTKhrY0HP6sJygWf-wd9CvvpsmN8wcowcQrvI9WjkqpMKQp3MEnZb3PywpV82cowc_dJKSpxbc-yW&amp;rn=c31858320f9edd93063daaeb5c4b4258&amp;spm=a1z10.5-b.w4011-25295428345.41.17026fa0qlqs4G" xr:uid="{71829057-A296-4489-9EC6-FA82043CF24A}"/>
-    <hyperlink ref="F5" r:id="rId4" display="https://detail.tmall.com/item.htm?abbucket=2&amp;id=668984438017&amp;ns=1&amp;pisk=gYcEF64oStC1lWgqfjVPgsxrl0VLL7-XTbZ7r40uRkq3A44uacmWJkgkv0lzj4HBJ8tdzwhZ0_1Bvp3la7NkcnOXG23Qw7xb7YvSKMU0ogA7xkqg9zwpfFs6G23L2wSklAAf4LtI3gXuq0VgIzzYZyVu-VYazzsuZk2ljO40j7qoqzbgjz4Px9quqFWguybhququjN48zMVuZ00M7zEg-biir25alJYlsWrsUO8Ypo03b_fVWzwHxVX5w_ea-Jlo8lus5fzULoy9uN_oaquoO5kVqp046jwSsVOP6WgqI54EqIx3sqDZlJle06Z-5Dh4tj-FOPwrvjyithCz5Y0sN72Gz_uscDe4o0JfpVV_k-DbpM54NXuiOPnPo9gLEAGLHXtGTSDxRWMojC5Emglf2PjRYbHFqTy3WPrX7FuAH_audye0YTB8ICUaceaCeTe3BPrX7NBReRxT7oTBi&amp;priceTId=213e367917381891117768651eb7a9&amp;skuId=4988894103512&amp;spm=a21n57.1.item.3.22d0340dlB9gUA&amp;utparam=%7B%22aplus_abtest%22%3A%220c383a5842c5f2f93401778954fef342%22%7D&amp;xxc=taobaoSearch" xr:uid="{0E16A982-207D-4FD7-A4BE-7DE62FB0C96B}"/>
-    <hyperlink ref="F6" r:id="rId5" xr:uid="{7FBB3596-8C34-40F4-AFA1-2FFE9B60DDEE}"/>
-    <hyperlink ref="F7" r:id="rId6" xr:uid="{1FE76F49-F361-4308-8081-5E19D7A8FC4F}"/>
-    <hyperlink ref="F8" r:id="rId7" display="https://detail.tmall.com/item.htm?abbucket=20&amp;id=43920214586&amp;ns=1&amp;pisk=gR8te46_nufshGM-QFohiQoginG3dDbw_G9_orbcID9ddISboc7GDZpCKFXMsN6bkKADSKYvgrCXGKlNnfoH_C7VlYDlk4Aw_IA80pTO12aBT_BbfDjsIC_0_YDorqn_OZHtEdVK8APCw__f1i6XOXCcNs6XhiaBO95VGR1b5Xhdg91bcPsbOW1RM5w6ht6IRsCfG16f1WZCLs_fhK_j9wG-4xBQ1t4v22HbQZDZ80nJJ1IOHPY0kd9urZBWg9ajFffNXlA1praXRH0AjQXxR8B2RKQ5lgFoBC7pSLCkI2a9eCtWh39IJPIefBLA4Euzw9T9MeIwxRiGdHdB7gxnByXwkOsJ5MmUpBOJ2IfRA7r99gWFJ39mGuB2t3IXqGytKtxktFspFv4p3iK6B6_54LYkysBbETC0fXhL0oS1TcBDUdg_tjQc9TctkorVYX5dEXhL0oSET6Bo6qE40MlF.&amp;priceTId=213e36c517383994625017887edf9f&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22f7ada5f1cf296bf680a317b2d42244ea%22%7D&amp;xxc=taobaoSearch&amp;sku_properties=5919063%3A6536025" xr:uid="{C02AC1E3-233B-4E7B-AC4E-4AFEAB13547C}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{5B37F600-9DE2-4AEA-96E7-A279D6B80EDB}"/>
+    <hyperlink ref="E3" r:id="rId2" display="https://detail.tmall.com/item.htm?abbucket=6&amp;id=663358716903&amp;pisk=gSEiq3GF3UvffHPJ6Wo1PT7ND-QKCdijOSKxMmhV8XlIXPLOCjz3FWXsDSeqiSVKOlBsMOO0i-2i7Akq7D-ECYJw0fy2nxPKbqatMfhmm-Nlp_IR2Rwscq5RwgnjxJCqVFl20IHeLxmmQlqGbiyscm5Dpn7RqRNPWXPo3xkFKxHv0APq_XlEOxD2QSlZ8Bkjhml4gSuETxMj3Fl2bB8EOYL2bfkwLBkxedlq_SyFKxGEgbZ2bbr4Ak5htVmzcY4uxA0iaJbB0nfnQQhuQ1tD0k4nSb--tn-4xA2dpUhkYilzPWzU7zvwvqnIt8MgGgtsbq4asvocmHog1Rrq-oCpsvaasku0vt_sdPy3m4ZfhFhTRS0uj2vfTviar5lLgKx8GcDSkrmcApGaPyFaYm9JRcU8eogzbGAS94M0ZYVMsgzy8U-J3nMFHk8XlVkIKb3i-vA2pFmSd9XHPmgZdACRK9YXhVkIK7WhKUNj7vMt7&amp;rn=3f9c2948bd3255c25dbbba65f1bf9b72&amp;spm=a1z10.5-b.w4011-25295428345.45.7ca8289cLqsyZo" xr:uid="{95147A8D-CAF1-4545-9FE2-3B467BD86C28}"/>
+    <hyperlink ref="E4" r:id="rId3" display="https://detail.tmall.com/item.htm?abbucket=6&amp;id=745189429142&amp;pisk=gCQxbx9jIDAXfaL3orZksBOSv2PuKNC2wt5ISdvmfTBRh9hcmKf61NBGFFx_3EbOeO6tSibDoha6etgMmNCZWC11QSJggufVgF8_KJYT-s5q15em-ZnjP01yOjO_qnwumOp3KJ43WoGWW-ehnDLCn0OpOFOXfdT7wCdXGFtXc3NJ1CDXCK61N7py_Ig6CFiWNBAjcFgXC4TWgI361mtXN39y1F91CFG4c-p-Gd0OvjLnPfZPpVg1yIK7xs95COFMGndAMLeQdaUeDp1XeVwEYk-9hB_QEmRpDOK5r1cnS3ffYORChxwv5_ddpBBYjfJAV6bDagytXpI1iMS14R3phMfFYhQ0K0fWlKKeLglTwFBPAHQy7filghOd3E_bExL9yB-GXt2r5KjdNTKhrY0HP6sJygWf-wd9CvvpsmN8wcowcQrvI9WjkqpMKQp3MEnZb3PywpV82cowc_dJKSpxbc-yW&amp;rn=c31858320f9edd93063daaeb5c4b4258&amp;spm=a1z10.5-b.w4011-25295428345.41.17026fa0qlqs4G" xr:uid="{71829057-A296-4489-9EC6-FA82043CF24A}"/>
+    <hyperlink ref="E5" r:id="rId4" display="https://detail.tmall.com/item.htm?abbucket=2&amp;id=668984438017&amp;ns=1&amp;pisk=gYcEF64oStC1lWgqfjVPgsxrl0VLL7-XTbZ7r40uRkq3A44uacmWJkgkv0lzj4HBJ8tdzwhZ0_1Bvp3la7NkcnOXG23Qw7xb7YvSKMU0ogA7xkqg9zwpfFs6G23L2wSklAAf4LtI3gXuq0VgIzzYZyVu-VYazzsuZk2ljO40j7qoqzbgjz4Px9quqFWguybhququjN48zMVuZ00M7zEg-biir25alJYlsWrsUO8Ypo03b_fVWzwHxVX5w_ea-Jlo8lus5fzULoy9uN_oaquoO5kVqp046jwSsVOP6WgqI54EqIx3sqDZlJle06Z-5Dh4tj-FOPwrvjyithCz5Y0sN72Gz_uscDe4o0JfpVV_k-DbpM54NXuiOPnPo9gLEAGLHXtGTSDxRWMojC5Emglf2PjRYbHFqTy3WPrX7FuAH_audye0YTB8ICUaceaCeTe3BPrX7NBReRxT7oTBi&amp;priceTId=213e367917381891117768651eb7a9&amp;skuId=4988894103512&amp;spm=a21n57.1.item.3.22d0340dlB9gUA&amp;utparam=%7B%22aplus_abtest%22%3A%220c383a5842c5f2f93401778954fef342%22%7D&amp;xxc=taobaoSearch" xr:uid="{0E16A982-207D-4FD7-A4BE-7DE62FB0C96B}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{7FBB3596-8C34-40F4-AFA1-2FFE9B60DDEE}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{1FE76F49-F361-4308-8081-5E19D7A8FC4F}"/>
+    <hyperlink ref="E8" r:id="rId7" display="https://detail.tmall.com/item.htm?abbucket=20&amp;id=43920214586&amp;ns=1&amp;pisk=gR8te46_nufshGM-QFohiQoginG3dDbw_G9_orbcID9ddISboc7GDZpCKFXMsN6bkKADSKYvgrCXGKlNnfoH_C7VlYDlk4Aw_IA80pTO12aBT_BbfDjsIC_0_YDorqn_OZHtEdVK8APCw__f1i6XOXCcNs6XhiaBO95VGR1b5Xhdg91bcPsbOW1RM5w6ht6IRsCfG16f1WZCLs_fhK_j9wG-4xBQ1t4v22HbQZDZ80nJJ1IOHPY0kd9urZBWg9ajFffNXlA1praXRH0AjQXxR8B2RKQ5lgFoBC7pSLCkI2a9eCtWh39IJPIefBLA4Euzw9T9MeIwxRiGdHdB7gxnByXwkOsJ5MmUpBOJ2IfRA7r99gWFJ39mGuB2t3IXqGytKtxktFspFv4p3iK6B6_54LYkysBbETC0fXhL0oS1TcBDUdg_tjQc9TctkorVYX5dEXhL0oSET6Bo6qE40MlF.&amp;priceTId=213e36c517383994625017887edf9f&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%22f7ada5f1cf296bf680a317b2d42244ea%22%7D&amp;xxc=taobaoSearch&amp;sku_properties=5919063%3A6536025" xr:uid="{C02AC1E3-233B-4E7B-AC4E-4AFEAB13547C}"/>
+    <hyperlink ref="E11" r:id="rId8" xr:uid="{7F05A493-E5C6-45F0-AF41-9BC3FFAC198D}"/>
+    <hyperlink ref="E15" r:id="rId9" xr:uid="{AA5F4F46-8A35-44BA-B75A-92677218D5DB}"/>
+    <hyperlink ref="E9" r:id="rId10" xr:uid="{7295C5AB-BAE9-4BCF-BAAF-896E943D6325}"/>
+    <hyperlink ref="E10" r:id="rId11" display="https://item.taobao.com/item.htm?id=809531552141&amp;ns=1&amp;pisk=gq8tep6_nuf6cqM-QFohi8WHLXhhHDAZIdR7otXgcpppG94m_NmVkKBp3OjG5O4AkIp2nKdq_s6XhKBDjD0k_C7VlYXxr4AwhLPaNdB1cwGfasFstGw91NP1lYDokkVCbAbXIvLRw2ZCa911Gi1s9w1AiP_fflgI9s10Coa6hXdCLsXb5s6bd61f6P_blZgQRs1Yflsff6_CLs_fhK_j9MG4ZxBQ1t4v2VjWZ4HFqraXJ1IIqBXBDnGc1GQJ69HSFe3PXTO1prHu2aSPC_TSKl5RXKIB-IVuoMA64K5WCRMOlBCJe_ptmSW9AQYGTHkYDTKXs3-XYxURC3Ay4iLiEkAC5OIPUHPx9ZpeVgLFuSZH_i1JQNTsKRQAJ_SDDdDUlOxJOpIk-J4lRQtdJg5WrUCAh8XRilGK9orVf6oOnLJs5WcAo6Bo6qE40MlF9TcK9orVYX5dEf330oSel&amp;priceTId=2150437317385084349456379eae0c&amp;skuId=5665172406995&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%22234b61a016079ef984d5a92ae51d05d9%22%7D&amp;xxc=ad_ztc" xr:uid="{AEAF3AD2-4262-4F27-8BAF-792436F9EE02}"/>
+    <hyperlink ref="E12" r:id="rId12" xr:uid="{85E6141B-215A-44E1-A9C3-50922778ED37}"/>
+    <hyperlink ref="E13" r:id="rId13" xr:uid="{A3B3ACE2-4624-40D4-A08A-575C8A24679D}"/>
+    <hyperlink ref="E14" r:id="rId14" xr:uid="{0591C9C3-F3D9-4BE1-9C39-2F12E94115C5}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{F9F22CAD-CA97-4D80-BA78-8C3BCD7ED349}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>